<commit_message>
Sync planning SharePoint : S21
</commit_message>
<xml_diff>
--- a/Plannings 2026 S21.xlsx
+++ b/Plannings 2026 S21.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F76A89A2-5C8C-43BB-810A-A43E91EB42FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{F76A89A2-5C8C-43BB-810A-A43E91EB42FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22C45F8B-D570-4703-9F47-4EE20EC3F5F7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -574,7 +574,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -607,6 +607,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -925,7 +937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1110,6 +1122,27 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1118,6 +1151,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFCCFF"/>
       <color rgb="FFCCFFFF"/>
       <color rgb="FFCC99FF"/>
     </mruColors>
@@ -6311,7 +6345,7 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="64" t="s">
         <v>14</v>
       </c>
       <c r="H7" s="22"/>
@@ -6323,7 +6357,7 @@
       <c r="D8" s="25"/>
       <c r="E8" s="25"/>
       <c r="F8" s="25"/>
-      <c r="G8" s="25" t="s">
+      <c r="G8" s="65" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="26"/>
@@ -6644,7 +6678,7 @@
       <c r="C30" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="19" t="s">
+      <c r="D30" s="62" t="s">
         <v>14</v>
       </c>
       <c r="E30" s="19"/>
@@ -6660,7 +6694,7 @@
       <c r="C31" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="63" t="s">
         <v>49</v>
       </c>
       <c r="E31" s="2"/>
@@ -6877,7 +6911,7 @@
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
-      <c r="G44" s="3" t="s">
+      <c r="G44" s="64" t="s">
         <v>14</v>
       </c>
       <c r="H44" s="22"/>
@@ -6889,7 +6923,7 @@
       <c r="D45" s="25"/>
       <c r="E45" s="25"/>
       <c r="F45" s="25"/>
-      <c r="G45" s="25" t="s">
+      <c r="G45" s="65" t="s">
         <v>74</v>
       </c>
       <c r="H45" s="26"/>
@@ -7050,7 +7084,7 @@
       <c r="E56" s="19"/>
       <c r="F56" s="19"/>
       <c r="G56" s="19"/>
-      <c r="H56" s="20" t="s">
+      <c r="H56" s="68" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7062,7 +7096,7 @@
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
-      <c r="H57" s="22" t="s">
+      <c r="H57" s="67" t="s">
         <v>87</v>
       </c>
     </row>
@@ -7188,7 +7222,7 @@
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
-      <c r="H67" s="32" t="s">
+      <c r="H67" s="66" t="s">
         <v>17</v>
       </c>
     </row>
@@ -7200,7 +7234,7 @@
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
-      <c r="H68" s="22" t="s">
+      <c r="H68" s="67" t="s">
         <v>94</v>
       </c>
     </row>
@@ -7260,7 +7294,7 @@
       <c r="C73" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="D73" s="19" t="s">
+      <c r="D73" s="62" t="s">
         <v>14</v>
       </c>
       <c r="E73" s="19"/>
@@ -7274,7 +7308,7 @@
       <c r="C74" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="D74" s="63" t="s">
         <v>98</v>
       </c>
       <c r="E74" s="2"/>
@@ -7510,7 +7544,7 @@
         <v>19</v>
       </c>
       <c r="C89" s="2"/>
-      <c r="D89" s="3" t="s">
+      <c r="D89" s="64" t="s">
         <v>14</v>
       </c>
       <c r="E89" s="2"/>
@@ -7528,7 +7562,7 @@
         <v>114</v>
       </c>
       <c r="C90" s="2"/>
-      <c r="D90" s="2" t="s">
+      <c r="D90" s="63" t="s">
         <v>115</v>
       </c>
       <c r="E90" s="2"/>
@@ -7544,10 +7578,10 @@
       <c r="A91" s="21"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
+      <c r="D91" s="63"/>
       <c r="E91" s="2"/>
       <c r="F91" s="2"/>
-      <c r="G91" s="3" t="s">
+      <c r="G91" s="64" t="s">
         <v>14</v>
       </c>
       <c r="H91" s="22"/>
@@ -7556,10 +7590,10 @@
       <c r="A92" s="21"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
+      <c r="D92" s="63"/>
       <c r="E92" s="2"/>
       <c r="F92" s="2"/>
-      <c r="G92" s="2" t="s">
+      <c r="G92" s="63" t="s">
         <v>118</v>
       </c>
       <c r="H92" s="22"/>
@@ -7568,7 +7602,7 @@
       <c r="A93" s="21"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
+      <c r="D93" s="63"/>
       <c r="E93" s="2"/>
       <c r="F93" s="2"/>
       <c r="G93" s="3" t="s">
@@ -7580,7 +7614,7 @@
       <c r="A94" s="23"/>
       <c r="B94" s="25"/>
       <c r="C94" s="25"/>
-      <c r="D94" s="25"/>
+      <c r="D94" s="65"/>
       <c r="E94" s="25"/>
       <c r="F94" s="25"/>
       <c r="G94" s="25" t="s">
@@ -7681,7 +7715,7 @@
       <c r="D101" s="19"/>
       <c r="E101" s="19"/>
       <c r="F101" s="19"/>
-      <c r="G101" s="19" t="s">
+      <c r="G101" s="62" t="s">
         <v>14</v>
       </c>
       <c r="H101" s="20"/>
@@ -7693,7 +7727,7 @@
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
       <c r="F102" s="2"/>
-      <c r="G102" s="2" t="s">
+      <c r="G102" s="63" t="s">
         <v>124</v>
       </c>
       <c r="H102" s="22"/>
@@ -8700,13 +8734,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA256E12-D58E-4CB0-A6BF-6C9C54BA964A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4442A821-9505-414A-9753-94FA89BA05D5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627E563C-1B39-4F2A-8AA0-EA74BDF79B40}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBC9276C-0F03-40F3-94EA-DEB664D2C6A7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD9D104E-E8A3-44EA-A87D-805054D515DC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AAF6256-C95F-4179-812B-DA083557110F}"/>
 </file>
</xml_diff>